<commit_message>
match excel import format to spec
</commit_message>
<xml_diff>
--- a/exampleRoster.xlsx
+++ b/exampleRoster.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kingsten/Desktop/chorus/seatingApp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A8647F7-8033-5A42-873F-DCEA119A1423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91E68A66-8D35-0A40-B0F7-F10776E05675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{C9C8D777-A17F-0D40-A2CF-B766D0ADF6F4}"/>
   </bookViews>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
-  <si>
-    <t>Name</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
   <si>
     <t>Part</t>
   </si>
@@ -62,9 +59,6 @@
     <t>T1</t>
   </si>
   <si>
-    <t>First Last</t>
-  </si>
-  <si>
     <t>A B</t>
   </si>
   <si>
@@ -78,6 +72,27 @@
   </si>
   <si>
     <t>I J</t>
+  </si>
+  <si>
+    <t>First</t>
+  </si>
+  <si>
+    <t>Last</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>hello</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>E</t>
   </si>
 </sst>
 </file>
@@ -450,86 +465,107 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F66CDFE6-EFC9-A840-B482-BC365CD277FF}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="D2" s="1">
+        <v>5.09</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="1">
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="1">
+        <v>5.0999999999999996</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="1">
         <v>5.09</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>11</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="1">
-        <v>5.0999999999999996</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="1">
-        <v>5.09</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="1">
+      <c r="D7" s="1">
         <v>5.0599999999999996</v>
       </c>
     </row>

</xml_diff>